<commit_message>
chore: ignore Office lock files (~$*) and untrack stray Word lock
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/פיתוח/דוגמאות/תחשיב זכויות אישי/DB למכתב תחשיב זכויות וחובות.xlsx
+++ b/פיתוח/דוגמאות/תחשיב זכויות אישי/DB למכתב תחשיב זכויות וחובות.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dfusb\Documents\מכונת מכתבים\תחשיב זכויות אישי\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dfusb\Documents\מכונת מכתבים\פיתוח\דוגמאות\תחשיב זכויות אישי\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6B5EED-203E-4B00-80B8-CF576416478D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C508B099-B1BF-4DEB-BD49-2E2BF2B5F3AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="972" windowWidth="17280" windowHeight="11988" xr2:uid="{230BCDDF-ECC3-443F-AB3B-8BCF8BF18170}"/>
+    <workbookView xWindow="1920" yWindow="972" windowWidth="17280" windowHeight="11988" xr2:uid="{230BCDDF-ECC3-443F-AB3B-8BCF8BF18170}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="35">
   <si>
     <t>סידורי</t>
   </si>
@@ -141,6 +141,9 @@
   </si>
   <si>
     <t>99-88-777</t>
+  </si>
+  <si>
+    <t>נקלט.ת</t>
   </si>
 </sst>
 </file>
@@ -867,7 +870,7 @@
         <v>33</v>
       </c>
       <c r="T4" s="8" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="U4" s="13">
         <v>70</v>

</xml_diff>